<commit_message>
Show company names in xls + pdf outputs
Add long_description field to RWLine and RTLine (default ""),
populated from Trade.description (broker-provided company name).
output_xls.py gets a dedicated "Azienda" column in both RW and RT
sheets. output_pdf.py renders the same in a 38mm column
(truncated at 32 chars) between Simbolo and Val./Acquisto.

Forex FIFO RT lines get a synthetic "Plusvalenza valutaria (FIFO
USD)" description instead of empty, so the EUR.USD rows in RT
also carry a human-readable label.

All five committed oracles (magnotta/2024, mosconi/2023-2024,
mascetti/2024-2025) regenerated to include the new field. Only
diff against the previous YAMLs is the new key — no computed
value shifts. examples/ regenerated likewise.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/magnotta/decaf_2024.xlsx
+++ b/examples/magnotta/decaf_2024.xlsx
@@ -647,27 +647,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -688,75 +689,80 @@
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
+          <t>Azienda</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
           <t>Descrizione</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Valuta</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Paese</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Quantita</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Acquisto</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Vendita</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Val. iniz. orig.</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Val. fin. orig.</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Cambio iniz.</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>Cambio fin.</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
         <is>
           <t>Val. iniz. EUR</t>
         </is>
       </c>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>Val. fin. EUR</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>Giorni</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>Quota %</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>IVAFE</t>
         </is>
@@ -778,57 +784,62 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>SAN GIORGIO INDUSTRIES SPA</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>SGRG (2024-01-17)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>500</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>2024-01-17</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2024-06-17</t>
         </is>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>752.1</v>
       </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
       <c r="M2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="P2" s="4" t="n">
         <v>752.1</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>153</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>100</v>
       </c>
-      <c r="R2" s="4" t="n">
+      <c r="S2" s="4" t="n">
         <v>0.63</v>
       </c>
     </row>
@@ -848,53 +859,58 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>BONTEMPI BISCOTTI INC</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>BGMP (2024-02-17)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>200</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>2024-02-17</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" s="4" t="n">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" s="4" t="n">
         <v>1100</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>1.0768</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>1.0389</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="O3" s="4" t="n">
         <v>1021.55</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="P3" s="4" t="n">
         <v>1155.07</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>319</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>100</v>
       </c>
-      <c r="R3" s="4" t="n">
+      <c r="S3" s="4" t="n">
         <v>2.01</v>
       </c>
     </row>
@@ -914,53 +930,58 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>CINQUE IMPERIA HOLDINGS SPA</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>CIMP (2024-03-05)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>100</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>2024-03-05</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" s="4" t="n">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" s="4" t="n">
         <v>1050</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>1250</v>
       </c>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
       <c r="M4" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>1050</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>1250</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>302</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>100</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>2.06</v>
       </c>
     </row>
@@ -974,56 +995,57 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Cash balance (USD)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>IE</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>7000</v>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" s="4" t="n">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>7000</v>
       </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
       <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
         <v>1.0389</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="O5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="P5" s="4" t="n">
         <v>6737.9</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>103</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>100</v>
       </c>
-      <c r="R5" s="4" t="n">
+      <c r="S5" s="4" t="n">
         <v>3.79</v>
       </c>
     </row>
     <row r="6">
-      <c r="R6" s="6" t="n"/>
+      <c r="S6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
@@ -1034,12 +1056,12 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>TOTALE</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
@@ -1047,7 +1069,8 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" s="4" t="n">
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" s="4" t="n">
         <v>8.49</v>
       </c>
     </row>
@@ -1062,21 +1085,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1092,50 +1116,55 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
+          <t>Azienda</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
           <t>Data acquisto</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Data vendita</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Quantita</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Corrispettivo EUR</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Costo EUR</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>+/- EUR</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Cambio BCE</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Forex</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>P/L broker</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>P/L broker EUR</t>
         </is>
@@ -1154,43 +1183,48 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>SAN GIORGIO INDUSTRIES SPA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>2024-06-15</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>2024-06-15</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>500</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>752.1</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>1000</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>-247.9</v>
       </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>-247.9</v>
       </c>
       <c r="L2" s="4" t="n">
         <v>-247.9</v>
       </c>
+      <c r="M2" s="4" t="n">
+        <v>-247.9</v>
+      </c>
     </row>
     <row r="3">
-      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr"/>
@@ -1199,12 +1233,13 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>NETTO</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>-247.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Release 0.3.1: art. 9 c. 2 per-lot ECB + settle-date RT + IBKR Closed Lots
- Per-lot ECB conversion on stock sales (art. 9 c. 2 TUIR)
- Settle-date tax-year assignment for RT (art. 68 TUIR)
- IBKR Closed Lots required for STK SELL; CASH SELL (forex) unaffected
- Pro-rata commission across per-lot Trades preserves forex_gains net USD
- QUERY_SETUP.md translated to Italian + Closed Lots steps added
- NORMATIVA.md: nuova §Conversione per-lotto, §Semplificazioni rimossa
- README §Limitazioni: 2 rimaste (obbligazioni, IVAFE black-list)
- jsdelivr README URLs pinned to @v0.3.1
- Examples regenerated
</commit_message>
<xml_diff>
--- a/examples/magnotta/decaf_2024.xlsx
+++ b/examples/magnotta/decaf_2024.xlsx
@@ -1188,12 +1188,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2024-06-15</t>
+          <t>2024-01-15</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2024-06-15</t>
+          <t>2024-06-17</t>
         </is>
       </c>
       <c r="F2" t="n">

</xml_diff>